<commit_message>
docs: align baseline requirements, design, and testing suite with confirmed stakeholder decisions (RD-023 to RD-029)
</commit_message>
<xml_diff>
--- a/Design/Data_Templates/Data_import_to_web.xlsx
+++ b/Design/Data_Templates/Data_import_to_web.xlsx
@@ -2,7 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R5c7f416b48f24cf3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R85a5f5cedfaf4d79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="2" r:id="Rb6f5bc48c3af4def"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Applicant" sheetId="3" r:id="R593489b8c9504751"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Loan History" sheetId="4" r:id="Ra12a4a492e464227"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scholarship History" sheetId="5" r:id="R2f272503aeeb4f27"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -125,19 +129,35 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="1">
+  <x:fonts count="2">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
       <x:name val="Calibri"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="2">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F6B78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F6B78"/>
+      </x:patternFill>
     </x:fill>
   </x:fills>
   <x:borders count="1">
@@ -146,10 +166,27 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="2">
+  <x:cellXfs count="9">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -550,4 +587,228 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="72" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
+      <x:c r="A1" s="8" t="str">
+        <x:v>Item</x:v>
+      </x:c>
+      <x:c r="B1" s="8" t="str">
+        <x:v>Confirmed Release 1 rule</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="7" t="str">
+        <x:v>Purpose</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="str">
+        <x:v>Workbook template for applicant, loan-history, and scholarship-history import.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="7" t="str">
+        <x:v>Application key</x:v>
+      </x:c>
+      <x:c r="B3" s="7" t="str">
+        <x:v>round_id + scholarship_type_id + student_id</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="7" t="str">
+        <x:v>Legacy support</x:v>
+      </x:c>
+      <x:c r="B4" s="7" t="str">
+        <x:v>Sheet1 is retained for transition only; new imports use the named sheets.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="7" t="str">
+        <x:v>Duplicate handling</x:v>
+      </x:c>
+      <x:c r="B5" s="7" t="str">
+        <x:v>Duplicate in file = Error; duplicate in database = Skip; never upsert.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="7" t="str">
+        <x:v>National ID</x:v>
+      </x:c>
+      <x:c r="B6" s="7" t="str">
+        <x:v>Out of Scope for Release 1.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="7" t="str">
+        <x:v>Amount input</x:v>
+      </x:c>
+      <x:c r="B7" s="7" t="str">
+        <x:v>Preset amount or Custom with a non-empty reason.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="14" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="22" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
+      <x:c r="A1" s="8" t="str">
+        <x:v>round_id</x:v>
+      </x:c>
+      <x:c r="B1" s="8" t="str">
+        <x:v>scholarship_type_id</x:v>
+      </x:c>
+      <x:c r="C1" s="8" t="str">
+        <x:v>student_id</x:v>
+      </x:c>
+      <x:c r="D1" s="8" t="str">
+        <x:v>prefix</x:v>
+      </x:c>
+      <x:c r="E1" s="8" t="str">
+        <x:v>first_name</x:v>
+      </x:c>
+      <x:c r="F1" s="8" t="str">
+        <x:v>last_name</x:v>
+      </x:c>
+      <x:c r="G1" s="8" t="str">
+        <x:v>faculty_code</x:v>
+      </x:c>
+      <x:c r="H1" s="8" t="str">
+        <x:v>program_code</x:v>
+      </x:c>
+      <x:c r="I1" s="8" t="str">
+        <x:v>study_level_code</x:v>
+      </x:c>
+      <x:c r="J1" s="8" t="str">
+        <x:v>year_level</x:v>
+      </x:c>
+      <x:c r="K1" s="8" t="str">
+        <x:v>semester</x:v>
+      </x:c>
+      <x:c r="L1" s="8" t="str">
+        <x:v>academic_year</x:v>
+      </x:c>
+      <x:c r="M1" s="8" t="str">
+        <x:v>application_status</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
+      <x:c r="A1" s="8" t="str">
+        <x:v>round_id</x:v>
+      </x:c>
+      <x:c r="B1" s="8" t="str">
+        <x:v>scholarship_type_id</x:v>
+      </x:c>
+      <x:c r="C1" s="8" t="str">
+        <x:v>student_id</x:v>
+      </x:c>
+      <x:c r="D1" s="8" t="str">
+        <x:v>loan_type_code</x:v>
+      </x:c>
+      <x:c r="E1" s="8" t="str">
+        <x:v>semester</x:v>
+      </x:c>
+      <x:c r="F1" s="8" t="str">
+        <x:v>academic_year</x:v>
+      </x:c>
+      <x:c r="G1" s="8" t="str">
+        <x:v>amount</x:v>
+      </x:c>
+      <x:c r="H1" s="8" t="str">
+        <x:v>currency</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
+      <x:c r="A1" s="8" t="str">
+        <x:v>round_id</x:v>
+      </x:c>
+      <x:c r="B1" s="8" t="str">
+        <x:v>scholarship_type_id</x:v>
+      </x:c>
+      <x:c r="C1" s="8" t="str">
+        <x:v>student_id</x:v>
+      </x:c>
+      <x:c r="D1" s="8" t="str">
+        <x:v>scholarship_code</x:v>
+      </x:c>
+      <x:c r="E1" s="8" t="str">
+        <x:v>semester</x:v>
+      </x:c>
+      <x:c r="F1" s="8" t="str">
+        <x:v>academic_year</x:v>
+      </x:c>
+      <x:c r="G1" s="8" t="str">
+        <x:v>amount</x:v>
+      </x:c>
+      <x:c r="H1" s="8" t="str">
+        <x:v>currency</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>